<commit_message>
Ops console improvements + scheduler Gophish-health guard
- console.js (+static mirror): client edit dialog, campaign status
  filter dropdown, employee email validation in setup, conditional
  launch button when no employees entered
- api/clients.py: guard /clients router with ops token (employee PII +
  write ops); add campaigns_per_year to create/update models
- main.py + api/ops.py: skip scheduled-campaign pass when Gophish is
  unreachable (background loop and manual /ops/run-scheduler now return
  503 instead of piling up zombie campaigns and burning LLM calls)
- tests: Phish Defend -> PhishDefend branding; fixture refresh
</commit_message>
<xml_diff>
--- a/test_filled_template.xlsx
+++ b/test_filled_template.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Employees'!$A$3:$F$102</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +42,13 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
       <color rgb="002F5496"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -54,7 +61,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +84,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
         <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,14 +122,16 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,16 +497,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -502,6 +517,7 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="8" customHeight="1"/>
     <row r="3" ht="50" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -842,7 +858,7 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • country: ISO 3166-1 alpha-2 code (e.g. DE, US, GB, FR).</t>
+          <t xml:space="preserve">  • country: ISO 3166-1 alpha-2 code (e.g. DE, US, GB, FR).  Only rows with data are imported.</t>
         </is>
       </c>
     </row>
@@ -867,10 +883,46 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Yellow cells are required.  Blue cells are examples (not imported).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="0" insertColumns="0" pivotTables="0" deleteRows="0" formatCells="0" formatRows="0" sort="0" password="CE4B"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="8">
+    <dataValidation sqref="A5:A24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Too Long" error="company_name must be 255 characters or fewer." type="textLength" operator="lessThanOrEqual">
+      <formula1>255</formula1>
+    </dataValidation>
+    <dataValidation sqref="B5:B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="contact_email must be 255 characters or fewer." type="textLength" operator="lessThanOrEqual">
+      <formula1>255</formula1>
+    </dataValidation>
+    <dataValidation sqref="C5:C24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="contact_name must be 255 characters or fewer." type="textLength" operator="lessThanOrEqual">
+      <formula1>255</formula1>
+    </dataValidation>
+    <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="textLength" operator="lessThanOrEqual">
+      <formula1>100</formula1>
+    </dataValidation>
+    <dataValidation sqref="E5:E24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Number" error="employee_count must be a whole number between 0 and 999999." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>999999</formula2>
+    </dataValidation>
+    <dataValidation sqref="F5:F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="country must be a 2-letter code (e.g. DE, US)." type="textLength" operator="lessThanOrEqual">
+      <formula1>10</formula1>
+    </dataValidation>
+    <dataValidation sqref="G5:G24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Number" error="campaigns_per_year must be between 1 and 365." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>365</formula2>
+    </dataValidation>
+    <dataValidation sqref="H5:H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Value" error="vishing_enabled must be TRUE, FALSE, or left blank." promptTitle="Vishing Enabled" prompt="Select TRUE or FALSE" type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -881,15 +933,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G118"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -899,6 +951,7 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="8" customHeight="1"/>
     <row r="3" ht="55" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -927,8 +980,7 @@
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>group
-(enum, optional, default='general')
-See dropdown</t>
+(enum, optional, default='general')</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1025,6 +1077,14 @@
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1954,104 +2014,121 @@
       <c r="E102" s="5" t="n"/>
       <c r="F102" s="5" t="n"/>
     </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>NOTES:</t>
+        </is>
+      </c>
+    </row>
     <row r="106">
-      <c r="A106" s="6" t="inlineStr">
-        <is>
-          <t>NOTES:</t>
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • email is required and must be unique per client (no duplicate emails within one company).</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • email is required and must be unique per client (no duplicate emails within one company).</t>
+          <t xml:space="preserve">  • name: employees’ real names — used for {.FirstName} personalization in emails. Stored hashed in DB.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • name: employees' real names — used for {{.FirstName}} personalization in emails.</t>
+          <t xml:space="preserve">  • group: determines which phishing scenarios the employee is likely to receive.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • group: determines which phishing scenarios the employee is likely to receive.</t>
+          <t xml:space="preserve">  •   • executive → CEO fraud, urgency alerts</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •   • executive → CEO fraud, urgency alerts</t>
+          <t xml:space="preserve">  •   • finance → invoice fraud, credential harvest</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •   • finance → invoice fraud, credential harvest</t>
+          <t xml:space="preserve">  •   • hr → credential harvest, malware attachment, shared docs</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •   • hr → credential harvest, malware attachment, shared docs</t>
+          <t xml:space="preserve">  •   • it_management → cloud notifications, voicemail, credential harvest</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •   • it_management → cloud notifications, voicemail, credential harvest</t>
+          <t xml:space="preserve">  •   • it_staff → malware attachment, credential harvest, shared docs</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •   • it_staff → malware attachment, credential harvest, shared docs</t>
+          <t xml:space="preserve">  •   • sales → LinkedIn messages, shared docs, urgency</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •   • sales → LinkedIn messages, shared docs, urgency</t>
+          <t xml:space="preserve">  •   • engineering → cloud notifications, voicemail, malware</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •   • engineering → cloud notifications, voicemail, malware</t>
+          <t xml:space="preserve">  •   • general → credential harvest, urgency, shared docs</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •   • general → credential harvest, urgency, shared docs</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Leave ID fields blank — they are auto-generated.</t>
+          <t xml:space="preserve">  • Only rows with a non-empty email column are imported.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="0" insertColumns="0" pivotTables="0" deleteRows="0" formatCells="0" formatRows="0" sort="0" password="CE4B"/>
+  <autoFilter ref="A3:F102"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="E4:E103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Group" error="Please select a valid group from the dropdown." promptTitle="Employee Group" prompt="Select employee group" type="list">
+  <dataValidations count="6">
+    <dataValidation sqref="A7:A102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Too Long" error="email must be 255 characters or fewer." type="textLength" operator="lessThanOrEqual">
+      <formula1>255</formula1>
+    </dataValidation>
+    <dataValidation sqref="B7:B102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="name must be 255 characters or fewer." type="textLength" operator="lessThanOrEqual">
+      <formula1>255</formula1>
+    </dataValidation>
+    <dataValidation sqref="C7:C102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="textLength" operator="lessThanOrEqual">
+      <formula1>100</formula1>
+    </dataValidation>
+    <dataValidation sqref="D7:D102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="textLength" operator="lessThanOrEqual">
+      <formula1>100</formula1>
+    </dataValidation>
+    <dataValidation sqref="E7:E102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Group" error="Please select a valid group from the dropdown." promptTitle="Employee Group" prompt="Select employee group" type="list">
       <formula1>"executive,finance,hr,it_management,it_staff,sales,engineering,general"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F7:F102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="linkedin_url must be 500 characters or fewer." type="textLength" operator="lessThanOrEqual">
+      <formula1>500</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>